<commit_message>
adding data points to Pos50 normal program
</commit_message>
<xml_diff>
--- a/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
+++ b/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Experiment 1 - Testing Fixation Time\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77566043-A885-4570-A786-6767984534C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6338F4B9-72FE-40E2-83C3-FBCCFECC87EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="945" windowWidth="18675" windowHeight="12975" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
+    <workbookView xWindow="9555" yWindow="1860" windowWidth="18675" windowHeight="12975" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
   </bookViews>
   <sheets>
     <sheet name="All Time Distributions" sheetId="2" r:id="rId1"/>
@@ -1134,6 +1134,9 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>4174</v>
+      </c>
       <c r="B52">
         <v>8552</v>
       </c>
@@ -1145,6 +1148,9 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>4752</v>
+      </c>
       <c r="B53">
         <v>2763</v>
       </c>
@@ -1156,6 +1162,9 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>1542</v>
+      </c>
       <c r="B54">
         <v>8498</v>
       </c>
@@ -1167,6 +1176,9 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>1582</v>
+      </c>
       <c r="B55">
         <v>6121</v>
       </c>
@@ -1178,6 +1190,9 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>4079</v>
+      </c>
       <c r="B56">
         <v>2994</v>
       </c>
@@ -1189,6 +1204,9 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>5095</v>
+      </c>
       <c r="B57">
         <v>3813</v>
       </c>
@@ -1200,6 +1218,9 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>5860</v>
+      </c>
       <c r="B58">
         <v>4216</v>
       </c>
@@ -1211,6 +1232,9 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>6549</v>
+      </c>
       <c r="B59">
         <v>6629</v>
       </c>
@@ -1222,6 +1246,9 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>9925</v>
+      </c>
       <c r="B60">
         <v>7943</v>
       </c>
@@ -1233,6 +1260,9 @@
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>5339</v>
+      </c>
       <c r="B61">
         <v>11518</v>
       </c>
@@ -1244,6 +1274,9 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>16535</v>
+      </c>
       <c r="B62">
         <v>3735</v>
       </c>
@@ -1255,6 +1288,9 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>4644</v>
+      </c>
       <c r="B63">
         <v>5533</v>
       </c>
@@ -1266,6 +1302,9 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>11016</v>
+      </c>
       <c r="B64">
         <v>10244</v>
       </c>
@@ -1276,7 +1315,10 @@
         <v>8129</v>
       </c>
     </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>6911</v>
+      </c>
       <c r="B65">
         <v>4378</v>
       </c>
@@ -1287,7 +1329,10 @@
         <v>5196</v>
       </c>
     </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>5222</v>
+      </c>
       <c r="B66">
         <v>4118</v>
       </c>
@@ -1298,7 +1343,10 @@
         <v>6901</v>
       </c>
     </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>4225</v>
+      </c>
       <c r="B67">
         <v>2042</v>
       </c>
@@ -1309,7 +1357,10 @@
         <v>6078</v>
       </c>
     </row>
-    <row r="68" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>17145</v>
+      </c>
       <c r="B68">
         <v>5618</v>
       </c>
@@ -1320,7 +1371,10 @@
         <v>5924</v>
       </c>
     </row>
-    <row r="69" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>5920</v>
+      </c>
       <c r="B69">
         <v>13135</v>
       </c>
@@ -1331,7 +1385,10 @@
         <v>6478</v>
       </c>
     </row>
-    <row r="70" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>3064</v>
+      </c>
       <c r="B70">
         <v>4003</v>
       </c>
@@ -1342,7 +1399,10 @@
         <v>10939</v>
       </c>
     </row>
-    <row r="71" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>4299</v>
+      </c>
       <c r="B71">
         <v>4159</v>
       </c>
@@ -1353,7 +1413,7 @@
         <v>2597</v>
       </c>
     </row>
-    <row r="72" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B72">
         <v>2037</v>
       </c>
@@ -1364,7 +1424,7 @@
         <v>4429</v>
       </c>
     </row>
-    <row r="73" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B73">
         <v>12801</v>
       </c>
@@ -1375,7 +1435,7 @@
         <v>9112</v>
       </c>
     </row>
-    <row r="74" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B74">
         <v>5698</v>
       </c>
@@ -1386,7 +1446,7 @@
         <v>3061</v>
       </c>
     </row>
-    <row r="75" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B75">
         <v>8958</v>
       </c>
@@ -1397,7 +1457,7 @@
         <v>9099</v>
       </c>
     </row>
-    <row r="76" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B76">
         <v>5455</v>
       </c>
@@ -1408,7 +1468,7 @@
         <v>3783</v>
       </c>
     </row>
-    <row r="77" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B77">
         <v>3134</v>
       </c>
@@ -1419,7 +1479,7 @@
         <v>6506</v>
       </c>
     </row>
-    <row r="78" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B78">
         <v>5022</v>
       </c>
@@ -1430,7 +1490,7 @@
         <v>3966</v>
       </c>
     </row>
-    <row r="79" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B79">
         <v>10345</v>
       </c>
@@ -1441,7 +1501,7 @@
         <v>5096</v>
       </c>
     </row>
-    <row r="80" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B80">
         <v>4880</v>
       </c>
@@ -1690,7 +1750,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14A4F54D-F9A8-4A57-B36F-2ADC46C86094}">
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -2256,6 +2316,226 @@
       </c>
       <c r="C51">
         <v>0.95194444444444448</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>4174</v>
+      </c>
+      <c r="B52">
+        <v>69.566666666666663</v>
+      </c>
+      <c r="C52">
+        <v>1.1594444444444445</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>4752</v>
+      </c>
+      <c r="B53">
+        <v>79.2</v>
+      </c>
+      <c r="C53">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>1542</v>
+      </c>
+      <c r="B54">
+        <v>25.7</v>
+      </c>
+      <c r="C54">
+        <v>0.42833333333333334</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>1582</v>
+      </c>
+      <c r="B55">
+        <v>26.366666666666667</v>
+      </c>
+      <c r="C55">
+        <v>0.43944444444444447</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>4079</v>
+      </c>
+      <c r="B56">
+        <v>67.983333333333334</v>
+      </c>
+      <c r="C56">
+        <v>1.1330555555555555</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>5095</v>
+      </c>
+      <c r="B57">
+        <v>84.916666666666671</v>
+      </c>
+      <c r="C57">
+        <v>1.4152777777777779</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>5860</v>
+      </c>
+      <c r="B58">
+        <v>97.666666666666671</v>
+      </c>
+      <c r="C58">
+        <v>1.6277777777777778</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>6549</v>
+      </c>
+      <c r="B59">
+        <v>109.15</v>
+      </c>
+      <c r="C59">
+        <v>1.8191666666666666</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>9925</v>
+      </c>
+      <c r="B60">
+        <v>165.41666666666666</v>
+      </c>
+      <c r="C60">
+        <v>2.7569444444444446</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>5339</v>
+      </c>
+      <c r="B61">
+        <v>88.983333333333334</v>
+      </c>
+      <c r="C61">
+        <v>1.4830555555555556</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>16535</v>
+      </c>
+      <c r="B62">
+        <v>275.58333333333331</v>
+      </c>
+      <c r="C62">
+        <v>4.5930555555555559</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>4644</v>
+      </c>
+      <c r="B63">
+        <v>77.400000000000006</v>
+      </c>
+      <c r="C63">
+        <v>1.29</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>11016</v>
+      </c>
+      <c r="B64">
+        <v>183.6</v>
+      </c>
+      <c r="C64">
+        <v>3.06</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>6911</v>
+      </c>
+      <c r="B65">
+        <v>115.18333333333334</v>
+      </c>
+      <c r="C65">
+        <v>1.9197222222222223</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>5222</v>
+      </c>
+      <c r="B66">
+        <v>87.033333333333331</v>
+      </c>
+      <c r="C66">
+        <v>1.4505555555555556</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>4225</v>
+      </c>
+      <c r="B67">
+        <v>70.416666666666671</v>
+      </c>
+      <c r="C67">
+        <v>1.1736111111111112</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>17145</v>
+      </c>
+      <c r="B68">
+        <v>285.75</v>
+      </c>
+      <c r="C68">
+        <v>4.7625000000000002</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>5920</v>
+      </c>
+      <c r="B69">
+        <v>98.666666666666671</v>
+      </c>
+      <c r="C69">
+        <v>1.6444444444444444</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>3064</v>
+      </c>
+      <c r="B70">
+        <v>51.06666666666667</v>
+      </c>
+      <c r="C70">
+        <v>0.85111111111111115</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>4299</v>
+      </c>
+      <c r="B71">
+        <v>71.650000000000006</v>
+      </c>
+      <c r="C71">
+        <v>1.1941666666666666</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding more normal equation data points
</commit_message>
<xml_diff>
--- a/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
+++ b/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Experiment 1 - Testing Fixation Time\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6338F4B9-72FE-40E2-83C3-FBCCFECC87EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6074201-39A5-4316-9F25-662940CA1104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9555" yWindow="1860" windowWidth="18675" windowHeight="12975" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
   </bookViews>
@@ -1414,6 +1414,9 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>5383</v>
+      </c>
       <c r="B72">
         <v>2037</v>
       </c>
@@ -1425,6 +1428,9 @@
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>5837</v>
+      </c>
       <c r="B73">
         <v>12801</v>
       </c>
@@ -1436,6 +1442,9 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>8102</v>
+      </c>
       <c r="B74">
         <v>5698</v>
       </c>
@@ -1447,6 +1456,9 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>2886</v>
+      </c>
       <c r="B75">
         <v>8958</v>
       </c>
@@ -1458,6 +1470,9 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>9160</v>
+      </c>
       <c r="B76">
         <v>5455</v>
       </c>
@@ -1469,6 +1484,9 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>1729</v>
+      </c>
       <c r="B77">
         <v>3134</v>
       </c>
@@ -1480,6 +1498,9 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>2198</v>
+      </c>
       <c r="B78">
         <v>5022</v>
       </c>
@@ -1491,6 +1512,9 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>13103</v>
+      </c>
       <c r="B79">
         <v>10345</v>
       </c>
@@ -1502,6 +1526,9 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>10956</v>
+      </c>
       <c r="B80">
         <v>4880</v>
       </c>
@@ -1512,7 +1539,10 @@
         <v>7606</v>
       </c>
     </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>3149</v>
+      </c>
       <c r="B81">
         <v>9557</v>
       </c>
@@ -1523,7 +1553,7 @@
         <v>5686</v>
       </c>
     </row>
-    <row r="82" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B82">
         <v>9578</v>
       </c>
@@ -1534,7 +1564,7 @@
         <v>4020</v>
       </c>
     </row>
-    <row r="83" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B83">
         <v>3413</v>
       </c>
@@ -1545,7 +1575,7 @@
         <v>11361</v>
       </c>
     </row>
-    <row r="84" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B84">
         <v>11804</v>
       </c>
@@ -1556,7 +1586,7 @@
         <v>4561</v>
       </c>
     </row>
-    <row r="85" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B85">
         <v>17299</v>
       </c>
@@ -1567,7 +1597,7 @@
         <v>4315</v>
       </c>
     </row>
-    <row r="86" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B86">
         <v>9940</v>
       </c>
@@ -1578,7 +1608,7 @@
         <v>6186</v>
       </c>
     </row>
-    <row r="87" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B87">
         <v>4185</v>
       </c>
@@ -1589,7 +1619,7 @@
         <v>9214</v>
       </c>
     </row>
-    <row r="88" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B88">
         <v>4214</v>
       </c>
@@ -1600,7 +1630,7 @@
         <v>21398</v>
       </c>
     </row>
-    <row r="89" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B89">
         <v>4853</v>
       </c>
@@ -1611,7 +1641,7 @@
         <v>1977</v>
       </c>
     </row>
-    <row r="90" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B90">
         <v>3857</v>
       </c>
@@ -1622,7 +1652,7 @@
         <v>10996</v>
       </c>
     </row>
-    <row r="91" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B91">
         <v>14386</v>
       </c>
@@ -1633,7 +1663,7 @@
         <v>6389</v>
       </c>
     </row>
-    <row r="92" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B92">
         <v>6377</v>
       </c>
@@ -1644,7 +1674,7 @@
         <v>9102</v>
       </c>
     </row>
-    <row r="93" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B93">
         <v>4942</v>
       </c>
@@ -1655,7 +1685,7 @@
         <v>6428</v>
       </c>
     </row>
-    <row r="94" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B94">
         <v>9667</v>
       </c>
@@ -1666,7 +1696,7 @@
         <v>4897</v>
       </c>
     </row>
-    <row r="95" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B95">
         <v>2532</v>
       </c>
@@ -1677,7 +1707,7 @@
         <v>4748</v>
       </c>
     </row>
-    <row r="96" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B96">
         <v>4231</v>
       </c>
@@ -1750,7 +1780,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14A4F54D-F9A8-4A57-B36F-2ADC46C86094}">
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -2536,6 +2566,116 @@
       </c>
       <c r="C71">
         <v>1.1941666666666666</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>5383</v>
+      </c>
+      <c r="B72">
+        <v>89.716666666666669</v>
+      </c>
+      <c r="C72">
+        <v>1.4952777777777777</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>5837</v>
+      </c>
+      <c r="B73">
+        <v>97.283333333333331</v>
+      </c>
+      <c r="C73">
+        <v>1.621388888888889</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>8102</v>
+      </c>
+      <c r="B74">
+        <v>135.03333333333333</v>
+      </c>
+      <c r="C74">
+        <v>2.2505555555555556</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>2886</v>
+      </c>
+      <c r="B75">
+        <v>48.1</v>
+      </c>
+      <c r="C75">
+        <v>0.80166666666666664</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>9160</v>
+      </c>
+      <c r="B76">
+        <v>152.66666666666666</v>
+      </c>
+      <c r="C76">
+        <v>2.5444444444444443</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>1729</v>
+      </c>
+      <c r="B77">
+        <v>28.816666666666666</v>
+      </c>
+      <c r="C77">
+        <v>0.4802777777777778</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>2198</v>
+      </c>
+      <c r="B78">
+        <v>36.633333333333333</v>
+      </c>
+      <c r="C78">
+        <v>0.61055555555555552</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>13103</v>
+      </c>
+      <c r="B79">
+        <v>218.38333333333333</v>
+      </c>
+      <c r="C79">
+        <v>3.6397222222222223</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>10956</v>
+      </c>
+      <c r="B80">
+        <v>182.6</v>
+      </c>
+      <c r="C80">
+        <v>3.0433333333333334</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>3149</v>
+      </c>
+      <c r="B81">
+        <v>52.483333333333334</v>
+      </c>
+      <c r="C81">
+        <v>0.87472222222222218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
finished Experiment 1 data collection
</commit_message>
<xml_diff>
--- a/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
+++ b/Experiment 1 - Testing Fixation Time/Time_for_Bac_Fix_Pos50_Start.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Moar Documents\GitHub\Bac_Evol_SSA\Experiment 1 - Testing Fixation Time\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6074201-39A5-4316-9F25-662940CA1104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B77D2C05-4028-4DB3-BA14-EFC4EDDC440E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9555" yWindow="1860" windowWidth="18675" windowHeight="12975" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
+    <workbookView xWindow="9900" yWindow="2205" windowWidth="18675" windowHeight="12975" xr2:uid="{C5D5DF43-D68A-448F-BEE9-BC751A2734F3}"/>
   </bookViews>
   <sheets>
     <sheet name="All Time Distributions" sheetId="2" r:id="rId1"/>
@@ -463,7 +463,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>13588</v>
+        <v>4174</v>
       </c>
       <c r="B4">
         <v>3898</v>
@@ -827,7 +827,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>29157</v>
+        <v>4174</v>
       </c>
       <c r="B30">
         <v>7969</v>
@@ -1554,6 +1554,9 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>3363</v>
+      </c>
       <c r="B82">
         <v>9578</v>
       </c>
@@ -1565,6 +1568,9 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>4437</v>
+      </c>
       <c r="B83">
         <v>3413</v>
       </c>
@@ -1576,6 +1582,9 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>7017</v>
+      </c>
       <c r="B84">
         <v>11804</v>
       </c>
@@ -1587,6 +1596,9 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>3118</v>
+      </c>
       <c r="B85">
         <v>17299</v>
       </c>
@@ -1598,6 +1610,9 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>1901</v>
+      </c>
       <c r="B86">
         <v>9940</v>
       </c>
@@ -1609,6 +1624,9 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>6500</v>
+      </c>
       <c r="B87">
         <v>4185</v>
       </c>
@@ -1620,6 +1638,9 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>8541</v>
+      </c>
       <c r="B88">
         <v>4214</v>
       </c>
@@ -1631,6 +1652,9 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>3962</v>
+      </c>
       <c r="B89">
         <v>4853</v>
       </c>
@@ -1642,6 +1666,9 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>4174</v>
+      </c>
       <c r="B90">
         <v>3857</v>
       </c>
@@ -1653,6 +1680,9 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>4752</v>
+      </c>
       <c r="B91">
         <v>14386</v>
       </c>
@@ -1664,6 +1694,9 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>1542</v>
+      </c>
       <c r="B92">
         <v>6377</v>
       </c>
@@ -1675,6 +1708,9 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>1582</v>
+      </c>
       <c r="B93">
         <v>4942</v>
       </c>
@@ -1686,6 +1722,9 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>4079</v>
+      </c>
       <c r="B94">
         <v>9667</v>
       </c>
@@ -1697,6 +1736,9 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>5095</v>
+      </c>
       <c r="B95">
         <v>2532</v>
       </c>
@@ -1708,6 +1750,9 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>5860</v>
+      </c>
       <c r="B96">
         <v>4231</v>
       </c>
@@ -1718,7 +1763,10 @@
         <v>6942</v>
       </c>
     </row>
-    <row r="97" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>6549</v>
+      </c>
       <c r="B97">
         <v>3207</v>
       </c>
@@ -1729,7 +1777,10 @@
         <v>7846</v>
       </c>
     </row>
-    <row r="98" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>5339</v>
+      </c>
       <c r="B98">
         <v>6991</v>
       </c>
@@ -1740,7 +1791,10 @@
         <v>10538</v>
       </c>
     </row>
-    <row r="99" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>2867</v>
+      </c>
       <c r="B99">
         <v>12951</v>
       </c>
@@ -1751,7 +1805,10 @@
         <v>11893</v>
       </c>
     </row>
-    <row r="100" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>2946</v>
+      </c>
       <c r="B100">
         <v>5939</v>
       </c>
@@ -1762,7 +1819,10 @@
         <v>9233</v>
       </c>
     </row>
-    <row r="101" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>3391</v>
+      </c>
       <c r="B101">
         <v>3549</v>
       </c>
@@ -1780,7 +1840,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14A4F54D-F9A8-4A57-B36F-2ADC46C86094}">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" bestFit="1" customWidth="1"/>
@@ -1822,13 +1882,13 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>13588</v>
+        <v>4174</v>
       </c>
       <c r="B4">
-        <v>226.46666666666667</v>
+        <v>69.566666666666663</v>
       </c>
       <c r="C4">
-        <v>3.7744444444444443</v>
+        <v>1.1594444444444445</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2108,13 +2168,13 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>29157</v>
+        <v>4174</v>
       </c>
       <c r="B30">
-        <v>485.95</v>
+        <v>69.566666666666663</v>
       </c>
       <c r="C30">
-        <v>8.0991666666666671</v>
+        <v>1.1594444444444445</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -2676,6 +2736,226 @@
       </c>
       <c r="C81">
         <v>0.87472222222222218</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>3363</v>
+      </c>
+      <c r="B82">
+        <v>56.05</v>
+      </c>
+      <c r="C82">
+        <v>0.9341666666666667</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>4437</v>
+      </c>
+      <c r="B83">
+        <v>73.95</v>
+      </c>
+      <c r="C83">
+        <v>1.2324999999999999</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>7017</v>
+      </c>
+      <c r="B84">
+        <v>116.95</v>
+      </c>
+      <c r="C84">
+        <v>1.9491666666666667</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>3118</v>
+      </c>
+      <c r="B85">
+        <v>51.966666666666669</v>
+      </c>
+      <c r="C85">
+        <v>0.86611111111111116</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>1901</v>
+      </c>
+      <c r="B86">
+        <v>31.683333333333334</v>
+      </c>
+      <c r="C86">
+        <v>0.5280555555555555</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>6500</v>
+      </c>
+      <c r="B87">
+        <v>108.33333333333333</v>
+      </c>
+      <c r="C87">
+        <v>1.8055555555555556</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88">
+        <v>8541</v>
+      </c>
+      <c r="B88">
+        <v>142.35</v>
+      </c>
+      <c r="C88">
+        <v>2.3725000000000001</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89">
+        <v>3962</v>
+      </c>
+      <c r="B89">
+        <v>66.033333333333331</v>
+      </c>
+      <c r="C89">
+        <v>1.1005555555555555</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90">
+        <v>4174</v>
+      </c>
+      <c r="B90">
+        <v>69.566666666666663</v>
+      </c>
+      <c r="C90">
+        <v>1.1594444444444445</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91">
+        <v>4752</v>
+      </c>
+      <c r="B91">
+        <v>79.2</v>
+      </c>
+      <c r="C91">
+        <v>1.32</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92">
+        <v>1542</v>
+      </c>
+      <c r="B92">
+        <v>25.7</v>
+      </c>
+      <c r="C92">
+        <v>0.42833333333333334</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93">
+        <v>1582</v>
+      </c>
+      <c r="B93">
+        <v>26.366666666666667</v>
+      </c>
+      <c r="C93">
+        <v>0.43944444444444447</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94">
+        <v>4079</v>
+      </c>
+      <c r="B94">
+        <v>67.983333333333334</v>
+      </c>
+      <c r="C94">
+        <v>1.1330555555555555</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95">
+        <v>5095</v>
+      </c>
+      <c r="B95">
+        <v>84.916666666666671</v>
+      </c>
+      <c r="C95">
+        <v>1.4152777777777779</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>5860</v>
+      </c>
+      <c r="B96">
+        <v>97.666666666666671</v>
+      </c>
+      <c r="C96">
+        <v>1.6277777777777778</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97">
+        <v>6549</v>
+      </c>
+      <c r="B97">
+        <v>109.15</v>
+      </c>
+      <c r="C97">
+        <v>1.8191666666666666</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98">
+        <v>5339</v>
+      </c>
+      <c r="B98">
+        <v>88.983333333333334</v>
+      </c>
+      <c r="C98">
+        <v>1.4830555555555556</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99">
+        <v>2867</v>
+      </c>
+      <c r="B99">
+        <v>47.783333333333331</v>
+      </c>
+      <c r="C99">
+        <v>0.79638888888888892</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100">
+        <v>2946</v>
+      </c>
+      <c r="B100">
+        <v>49.1</v>
+      </c>
+      <c r="C100">
+        <v>0.81833333333333336</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101">
+        <v>3391</v>
+      </c>
+      <c r="B101">
+        <v>56.516666666666666</v>
+      </c>
+      <c r="C101">
+        <v>0.94194444444444447</v>
       </c>
     </row>
   </sheetData>

</xml_diff>